<commit_message>
#16 Client BOM added.
</commit_message>
<xml_diff>
--- a/Design-Files/photo_frame-v1.2/Deliverables/BOM/Client-BOM_photo_frame-v1.2.xlsx
+++ b/Design-Files/photo_frame-v1.2/Deliverables/BOM/Client-BOM_photo_frame-v1.2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\umarkhan-photoframe\Design-Files\photo_frame-v1.2\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="252">
   <si>
     <t>#</t>
   </si>
@@ -408,12 +408,6 @@
     <t>AFC24-S40FIC-00</t>
   </si>
   <si>
-    <t>Voltlink Target</t>
-  </si>
-  <si>
-    <t>TYPE-C-31-M-12_</t>
-  </si>
-  <si>
     <t>XAL1580-202MED</t>
   </si>
   <si>
@@ -441,9 +435,6 @@
     <t>B3U-1000P</t>
   </si>
   <si>
-    <t>MT-0-102-C003-N003-RS*</t>
-  </si>
-  <si>
     <t>38-SMD Module</t>
   </si>
   <si>
@@ -660,9 +651,6 @@
     <t>Diodes Incorporated</t>
   </si>
   <si>
-    <t>Comment</t>
-  </si>
-  <si>
     <t>10uF</t>
   </si>
   <si>
@@ -708,12 +696,6 @@
     <t>2uH</t>
   </si>
   <si>
-    <t>RED</t>
-  </si>
-  <si>
-    <t>S8050</t>
-  </si>
-  <si>
     <t>10K</t>
   </si>
   <si>
@@ -762,14 +744,44 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>#Column Name Error:' Remarks</t>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>LCD</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> IPS ILI9488 No Touch</t>
+  </si>
+  <si>
+    <t>Aliexpress Note: Selection from link options: IPS ILI9488 No Touch</t>
+  </si>
+  <si>
+    <t>USB cable and Adapter</t>
+  </si>
+  <si>
+    <t>UGREEN 140W USB C Charger, Mac Book Pro Charger Nexode PD3.1 PPS 3-Port Foldable GaN Fast Laptop Wall Charger Power Adapter for MacBook Pro 16'', iPhone 16/15, Chromebook (with 240W Cable)</t>
+  </si>
+  <si>
+    <t>USB C Charger</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -810,6 +822,34 @@
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -925,10 +965,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -968,8 +1011,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1255,22 +1314,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K52"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="15.75" thickBot="1">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1283,7 +1342,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1301,28 +1360,30 @@
         <v>119</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>213</v>
+        <v>241</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" thickBot="1">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="12"/>
+      <c r="C3" s="12" t="s">
+        <v>2</v>
+      </c>
       <c r="D3" s="7" t="s">
         <v>22</v>
       </c>
@@ -1333,26 +1394,28 @@
         <v>120</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="J3" s="7">
         <v>4</v>
       </c>
       <c r="K3" s="7"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15.75" thickBot="1">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
         <f t="shared" ref="B4:B50" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="13"/>
+      <c r="C4" s="12" t="s">
+        <v>2</v>
+      </c>
       <c r="D4" s="9" t="s">
         <v>23</v>
       </c>
@@ -1363,20 +1426,20 @@
         <v>121</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="J4" s="9">
         <v>4</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="36.75" thickBot="1">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1395,26 +1458,28 @@
         <v>120</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
       </c>
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="13"/>
+      <c r="C6" s="12" t="s">
+        <v>2</v>
+      </c>
       <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
@@ -1425,27 +1490,27 @@
         <v>122</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>26</v>
@@ -1457,26 +1522,26 @@
         <v>120</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" thickBot="1">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
@@ -1489,27 +1554,27 @@
         <v>123</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15.75" thickBot="1">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
         <v>7</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>28</v>
@@ -1521,26 +1586,26 @@
         <v>121</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15.75" thickBot="1">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
@@ -1553,27 +1618,27 @@
         <v>120</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
       </c>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15.75" thickBot="1">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
         <v>9</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>30</v>
@@ -1585,27 +1650,27 @@
         <v>121</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
       <c r="K11" s="7"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15.75" thickBot="1">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>3</v>
+      <c r="C12" s="12" t="s">
+        <v>2</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>31</v>
@@ -1617,27 +1682,27 @@
         <v>120</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15.75" thickBot="1">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>32</v>
@@ -1649,27 +1714,27 @@
         <v>121</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
       </c>
       <c r="K13" s="7"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15.75" thickBot="1">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="13" t="s">
-        <v>3</v>
+      <c r="C14" s="12" t="s">
+        <v>2</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>33</v>
@@ -1681,27 +1746,27 @@
         <v>121</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
       <c r="K14" s="9"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15.75" thickBot="1">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>34</v>
@@ -1713,26 +1778,26 @@
         <v>121</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="36.75" thickBot="1">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D16" s="9" t="s">
@@ -1741,24 +1806,24 @@
       <c r="E16" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="F16" s="9" t="s">
-        <v>124</v>
+      <c r="F16" s="7" t="s">
+        <v>243</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>124</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="J16" s="9">
         <v>10</v>
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15.75" thickBot="1">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
@@ -1777,20 +1842,20 @@
         <v>121</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
       </c>
       <c r="K17" s="7"/>
     </row>
-    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="24.75" thickBot="1">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1809,20 +1874,20 @@
         <v>125</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>160</v>
+        <v>244</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="36.75" thickBot="1">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
@@ -1841,20 +1906,20 @@
         <v>126</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>161</v>
+        <v>195</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>244</v>
       </c>
       <c r="J19" s="7">
         <v>3</v>
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="24.75" thickBot="1">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
@@ -1873,20 +1938,20 @@
         <v>127</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>162</v>
+        <v>244</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="72.75" thickBot="1">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
@@ -1902,23 +1967,23 @@
         <v>89</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>128</v>
+        <v>243</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>128</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>128</v>
+        <v>197</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>244</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
       </c>
       <c r="K21" s="7"/>
     </row>
-    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="36.75" thickBot="1">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
@@ -1933,24 +1998,24 @@
       <c r="E22" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="9" t="s">
-        <v>129</v>
+      <c r="F22" s="7" t="s">
+        <v>243</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>129</v>
+        <v>244</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="24.75" thickBot="1">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1966,23 +2031,23 @@
         <v>91</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>130</v>
+        <v>243</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>164</v>
+        <v>199</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>244</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
       </c>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="15.75" thickBot="1">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1997,24 +2062,24 @@
       <c r="E24" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="F24" s="9" t="s">
-        <v>131</v>
+      <c r="F24" s="7" t="s">
+        <v>243</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="409.6" thickBot="1">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -2030,23 +2095,23 @@
         <v>93</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>132</v>
+        <v>243</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>132</v>
+        <v>244</v>
       </c>
       <c r="J25" s="7">
         <v>190</v>
       </c>
       <c r="K25" s="7"/>
     </row>
-    <row r="26" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="24.75" thickBot="1">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -2062,23 +2127,23 @@
         <v>94</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>229</v>
+        <v>202</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
       </c>
       <c r="K26" s="9"/>
     </row>
-    <row r="27" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="24.75" thickBot="1">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f>ROW(B27) - ROW($B$2)</f>
@@ -2094,23 +2159,23 @@
         <v>95</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>230</v>
+        <v>244</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="15.75" thickBot="1">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
@@ -2126,23 +2191,23 @@
         <v>96</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>167</v>
+        <v>204</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
       </c>
       <c r="K28" s="9"/>
     </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="15.75" thickBot="1">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
@@ -2158,23 +2223,23 @@
         <v>97</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>168</v>
+        <v>244</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
       </c>
       <c r="K29" s="7"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="15.75" thickBot="1">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
@@ -2190,23 +2255,23 @@
         <v>98</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="J30" s="9">
         <v>6</v>
       </c>
       <c r="K30" s="9"/>
     </row>
-    <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="15.75" thickBot="1">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
@@ -2222,23 +2287,23 @@
         <v>99</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="15.75" thickBot="1">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2254,23 +2319,23 @@
         <v>100</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
       <c r="K32" s="9"/>
     </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="15.75" thickBot="1">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
@@ -2286,23 +2351,23 @@
         <v>101</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="15.75" thickBot="1">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
@@ -2318,23 +2383,23 @@
         <v>102</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
       </c>
       <c r="K34" s="9"/>
     </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="15.75" thickBot="1">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
         <f>ROW(B35) - ROW($B$2)</f>
@@ -2350,23 +2415,23 @@
         <v>103</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
       </c>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="15.75" thickBot="1">
       <c r="A36" s="1"/>
       <c r="B36" s="11">
         <f t="shared" si="0"/>
@@ -2382,23 +2447,23 @@
         <v>104</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
       </c>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="15.75" thickBot="1">
       <c r="A37" s="1"/>
       <c r="B37" s="11">
         <f>ROW(B37) - ROW($B$2)</f>
@@ -2414,23 +2479,23 @@
         <v>105</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
       </c>
       <c r="K37" s="7"/>
     </row>
-    <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="15.75" thickBot="1">
       <c r="A38" s="1"/>
       <c r="B38" s="11">
         <f t="shared" si="0"/>
@@ -2446,23 +2511,23 @@
         <v>106</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
       </c>
       <c r="K38" s="9"/>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="15.75" thickBot="1">
       <c r="A39" s="1"/>
       <c r="B39" s="11">
         <f>ROW(B39) - ROW($B$2)</f>
@@ -2478,23 +2543,23 @@
         <v>107</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
       </c>
       <c r="K39" s="7"/>
     </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="15.75" thickBot="1">
       <c r="A40" s="1"/>
       <c r="B40" s="11">
         <f t="shared" si="0"/>
@@ -2510,23 +2575,23 @@
         <v>108</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="J40" s="9">
         <v>2</v>
       </c>
       <c r="K40" s="9"/>
     </row>
-    <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15.75" thickBot="1">
       <c r="A41" s="1"/>
       <c r="B41" s="11">
         <f>ROW(B41) - ROW($B$2)</f>
@@ -2542,23 +2607,23 @@
         <v>109</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
       </c>
       <c r="K41" s="7"/>
     </row>
-    <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="15.75" thickBot="1">
       <c r="A42" s="1"/>
       <c r="B42" s="11">
         <f t="shared" si="0"/>
@@ -2574,23 +2639,23 @@
         <v>110</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="15.75" thickBot="1">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
@@ -2606,23 +2671,23 @@
         <v>111</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="J43" s="7">
         <v>1</v>
       </c>
       <c r="K43" s="7"/>
     </row>
-    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="15.75" thickBot="1">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
@@ -2638,23 +2703,23 @@
         <v>112</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
       </c>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="15.75" thickBot="1">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f>ROW(B45) - ROW($B$2)</f>
@@ -2670,23 +2735,23 @@
         <v>113</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>139</v>
+        <v>243</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>139</v>
+        <v>244</v>
       </c>
       <c r="J45" s="7">
         <v>2</v>
       </c>
       <c r="K45" s="7"/>
     </row>
-    <row r="46" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="36.75" thickBot="1">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f t="shared" si="0"/>
@@ -2701,24 +2766,24 @@
       <c r="E46" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="F46" s="9" t="s">
-        <v>140</v>
+      <c r="F46" s="7" t="s">
+        <v>243</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="I46" s="10" t="s">
-        <v>184</v>
+        <v>206</v>
+      </c>
+      <c r="I46" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
       </c>
       <c r="K46" s="9"/>
     </row>
-    <row r="47" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="15.75" thickBot="1">
       <c r="A47" s="1"/>
       <c r="B47" s="11">
         <f>ROW(B47) - ROW($B$2)</f>
@@ -2734,23 +2799,23 @@
         <v>115</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>185</v>
+        <v>244</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
       </c>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="15.75" thickBot="1">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -2766,23 +2831,23 @@
         <v>116</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="I48" s="10" t="s">
-        <v>186</v>
+        <v>208</v>
+      </c>
+      <c r="I48" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
       </c>
       <c r="K48" s="9"/>
     </row>
-    <row r="49" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="36.75" thickBot="1">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
@@ -2798,23 +2863,23 @@
         <v>117</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>187</v>
+        <v>244</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
       </c>
       <c r="K49" s="7"/>
     </row>
-    <row r="50" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="36.75" thickBot="1">
       <c r="A50" s="1"/>
       <c r="B50" s="11">
         <f t="shared" si="0"/>
@@ -2830,27 +2895,97 @@
         <v>118</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="I50" s="10" t="s">
-        <v>188</v>
+        <v>204</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
       </c>
       <c r="K50" s="9"/>
+    </row>
+    <row r="51" spans="1:11" ht="45.75" thickBot="1">
+      <c r="B51" s="15">
+        <f t="shared" ref="B51:B52" si="1">ROW(B51)-ROW($B$2)</f>
+        <v>49</v>
+      </c>
+      <c r="C51" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="D51" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>247</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="G51" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="H51" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I51" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="J51" s="17">
+        <v>1</v>
+      </c>
+      <c r="K51" s="19" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="72.75" thickBot="1">
+      <c r="B52" s="15">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="C52" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="D52" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="E52" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="F52" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="G52" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="H52" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="I52" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="J52" s="17">
+        <v>1</v>
+      </c>
+      <c r="K52" s="19" t="s">
+        <v>251</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K51" r:id="rId1"/>
+    <hyperlink ref="K52" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>